<commit_message>
Seed cited startup_benchmarks table + surface benchmark band in Phase 0
- scripts/seed_startup_benchmarks.py: new startup_benchmarks table (idempotent),
  7 boutique-hotel rows with low/typical/high bands + cited sources
  (Fáilte Ireland Hotel Survey 2024, USALI, HotelData 2025)
- startup_build.py: Phase 0 now renders a cited benchmark band read from the
  table; Assumptions SOURCES updated with the specific Fáilte Ireland figures
- research/hotel_benchmarks.md: full benchmark reference with citations
- Confirms seed assumptions (ADR EUR135, occ 72%, RevPAR EUR97) sit inside the
  published 4-star bands. All 12 workbooks still pass validation.
</commit_message>
<xml_diff>
--- a/asset-forge/products/industries/hospitality/boutique-hotel-4star/00_Market_Validation.xlsx
+++ b/asset-forge/products/industries/hospitality/boutique-hotel-4star/00_Market_Validation.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="166" formatCode="#,##0\ &quot;€&quot;"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,6 +99,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="7">
@@ -184,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -230,6 +236,19 @@
     <xf numFmtId="3" fontId="6" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="8" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -255,7 +274,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -679,11 +697,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
-    <col width="42.1" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
     <col width="34.6" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -866,7 +884,7 @@
     <row r="13" ht="24" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>COMPETITOR MATRIX</t>
+          <t>INDUSTRY BENCHMARK BAND (CITED)</t>
         </is>
       </c>
       <c r="C13" s="5" t="n"/>
@@ -878,162 +896,197 @@
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Competitor</t>
+          <t>Metric</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Rooms</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Est. ADR €</t>
+          <t>Typical</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Rating /5</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Key strength</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Your edge vs them</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="19" customHeight="1">
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>The Harbour Townhouse</t>
+          <t>ADR — 4★ average daily rate</t>
         </is>
       </c>
       <c r="C15" s="18" t="n">
-        <v>28</v>
-      </c>
-      <c r="D15" s="19" t="n">
-        <v>145</v>
-      </c>
-      <c r="E15" s="20" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Sea views, spa</t>
-        </is>
-      </c>
-      <c r="G15" s="21" t="n"/>
-    </row>
-    <row r="16" ht="19" customHeight="1">
+        <v>127</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>144</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>241</v>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Fáilte Ireland Hotel Survey Nov/Dec 2024 (4★ ADR €143.50–€144.49; county range €127–€241)</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>City Mews Boutique</t>
-        </is>
-      </c>
-      <c r="C16" s="18" t="n">
-        <v>19</v>
-      </c>
-      <c r="D16" s="19" t="n">
-        <v>128</v>
-      </c>
-      <c r="E16" s="20" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="F16" s="14" t="inlineStr">
-        <is>
-          <t>Design-led, central</t>
-        </is>
-      </c>
-      <c r="G16" s="21" t="n"/>
-    </row>
-    <row r="17" ht="19" customHeight="1">
+          <t>Occupancy — 4★</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="n">
+        <v>0.602</v>
+      </c>
+      <c r="D16" s="21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E16" s="21" t="n">
+        <v>0.741</v>
+      </c>
+      <c r="F16" s="22" t="inlineStr">
+        <is>
+          <t>Fáilte Ireland Hotel Survey 2024 (4★ occ 60.2% Dec → 74.1% Nov)</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>The Old Mill Hotel</t>
+          <t>RevPAR — 4★</t>
         </is>
       </c>
       <c r="C17" s="18" t="n">
-        <v>32</v>
-      </c>
-      <c r="D17" s="19" t="n">
-        <v>119</v>
-      </c>
-      <c r="E17" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Free parking, events</t>
-        </is>
-      </c>
-      <c r="G17" s="21" t="n"/>
-    </row>
-    <row r="18" ht="19" customHeight="1">
+        <v>86.42</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>97</v>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>107.07</v>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>Fáilte Ireland Hotel Survey 2024 (4★ RevPAR €86.42 Dec → €107.07 Nov)</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Riverside Guesthouse</t>
-        </is>
-      </c>
-      <c r="C18" s="18" t="n">
-        <v>12</v>
-      </c>
-      <c r="D18" s="19" t="n">
-        <v>99</v>
-      </c>
-      <c r="E18" s="20" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F18" s="14" t="inlineStr">
-        <is>
-          <t>Owner-hosted, breakfast</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="n"/>
-    </row>
-    <row r="19"/>
-    <row r="20" ht="19" customHeight="1">
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>Competitor avg ADR</t>
-        </is>
-      </c>
-      <c r="D20" s="22">
-        <f>AVERAGE(D15:D18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="19" customHeight="1">
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>Your planned ADR</t>
-        </is>
-      </c>
-      <c r="D21" s="22">
-        <f>'Assumptions'!D6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Your ADR vs market</t>
-        </is>
-      </c>
-      <c r="D22" s="23">
-        <f>IFERROR('Assumptions'!D6/AVERAGE(D15:D18)-1,"")</f>
-        <v/>
+          <t>Labour cost (% of total revenue)</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D18" s="21" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="E18" s="21" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F18" s="22" t="inlineStr">
+        <is>
+          <t>Hospitality labour benchmark 25–35% of revenue; US long-run 31.2% (Mandelbaum/CBRE; altametrics)</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>F&amp;B cost (% of F&amp;B revenue)</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D19" s="21" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>USALI F&amp;B cost-of-sales; academic luxury 17.86% (US) – 23.87% (Asia)</t>
+        </is>
+      </c>
+      <c r="G19" s="20" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Rooms dept cost ex-payroll (% of rooms rev)</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D20" s="21" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E20" s="21" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="F20" s="22" t="inlineStr">
+        <is>
+          <t>USALI rooms departmental expense (rooms expense ~27–28% incl. labour; ex-labour ~8–18%)</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>GOP margin (% of total revenue)</t>
+        </is>
+      </c>
+      <c r="C21" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D21" s="21" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="E21" s="21" t="n">
+        <v>0.383</v>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>HotelData Q4-2025 full-year GOP margin 38.3%; academic luxury 33.2–36.7%</t>
+        </is>
+      </c>
+      <c r="G21" s="20" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Compare your Assumptions against these published bands; stay within Typical–High to be credible to lenders/grant assessors.</t>
+        </is>
       </c>
     </row>
     <row r="23"/>
     <row r="24" ht="24" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>LOCATION SCORING (WEIGHTED)</t>
+          <t>COMPETITOR MATRIX</t>
         </is>
       </c>
       <c r="C24" s="5" t="n"/>
@@ -1045,251 +1098,427 @@
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Factor</t>
+          <t>Competitor</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Weight</t>
+          <t>Rooms</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Score /10</t>
+          <t>Est. ADR €</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Weighted</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr"/>
-      <c r="G25" s="6" t="inlineStr"/>
+          <t>Rating /5</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Key strength</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Your edge vs them</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="19" customHeight="1">
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Footfall / visibility</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D26" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="E26" s="24">
-        <f>C26*D26</f>
-        <v/>
-      </c>
-      <c r="F26" s="8" t="n"/>
-      <c r="G26" s="8" t="n"/>
+          <t>The Harbour Townhouse</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="n">
+        <v>28</v>
+      </c>
+      <c r="D26" s="24" t="n">
+        <v>145</v>
+      </c>
+      <c r="E26" s="25" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Sea views, spa</t>
+        </is>
+      </c>
+      <c r="G26" s="26" t="n"/>
     </row>
     <row r="27" ht="19" customHeight="1">
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>Transport access</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D27" s="18" t="n">
-        <v>7</v>
-      </c>
-      <c r="E27" s="24">
-        <f>C27*D27</f>
-        <v/>
-      </c>
-      <c r="F27" s="14" t="n"/>
-      <c r="G27" s="14" t="n"/>
+          <t>City Mews Boutique</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="D27" s="24" t="n">
+        <v>128</v>
+      </c>
+      <c r="E27" s="25" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>Design-led, central</t>
+        </is>
+      </c>
+      <c r="G27" s="26" t="n"/>
     </row>
     <row r="28" ht="19" customHeight="1">
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Nearby demand drivers</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D28" s="18" t="n">
-        <v>9</v>
-      </c>
-      <c r="E28" s="24">
-        <f>C28*D28</f>
-        <v/>
-      </c>
-      <c r="F28" s="8" t="n"/>
-      <c r="G28" s="8" t="n"/>
+          <t>The Old Mill Hotel</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="D28" s="24" t="n">
+        <v>119</v>
+      </c>
+      <c r="E28" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Free parking, events</t>
+        </is>
+      </c>
+      <c r="G28" s="26" t="n"/>
     </row>
     <row r="29" ht="19" customHeight="1">
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>Competition density</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D29" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="E29" s="24">
-        <f>C29*D29</f>
-        <v/>
-      </c>
-      <c r="F29" s="14" t="n"/>
-      <c r="G29" s="14" t="n"/>
-    </row>
-    <row r="30" ht="19" customHeight="1">
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Lease cost vs ADR</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D30" s="18" t="n">
-        <v>7</v>
-      </c>
-      <c r="E30" s="24">
-        <f>C30*D30</f>
-        <v/>
-      </c>
-      <c r="F30" s="8" t="n"/>
-      <c r="G30" s="8" t="n"/>
-    </row>
+          <t>Riverside Guesthouse</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="D29" s="24" t="n">
+        <v>99</v>
+      </c>
+      <c r="E29" s="25" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Owner-hosted, breakfast</t>
+        </is>
+      </c>
+      <c r="G29" s="26" t="n"/>
+    </row>
+    <row r="30"/>
     <row r="31" ht="19" customHeight="1">
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Planning / fit-out ease</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D31" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="E31" s="24">
-        <f>C31*D31</f>
-        <v/>
-      </c>
-      <c r="F31" s="14" t="n"/>
-      <c r="G31" s="14" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="25" t="inlineStr">
-        <is>
-          <t>Location score / 10</t>
-        </is>
-      </c>
-      <c r="E32" s="26">
-        <f>SUM(E26:E31)</f>
-        <v/>
-      </c>
-      <c r="F32" s="27">
-        <f>IF(E32="","",IF(E32&gt;=7,"🟢 On target",IF(E32&gt;=5,"🟡 Watch","🔴 Action")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33"/>
-    <row r="34" ht="24" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>PHASE 0 GO / NO-GO GATE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="5" t="n"/>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
-    </row>
-    <row r="35" ht="19" customHeight="1">
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>SOM room-nights within capacity</t>
-        </is>
-      </c>
-      <c r="C35" s="28" t="n"/>
-      <c r="D35" s="28" t="n"/>
-      <c r="E35" s="28" t="n"/>
-      <c r="F35" s="29">
-        <f>IF(F8&lt;= ('Assumptions'!D5*365),"PASS","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="G35" s="8" t="n"/>
-    </row>
-    <row r="36" ht="19" customHeight="1">
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>ADR competitive (within ±15% of market)</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="n"/>
-      <c r="D36" s="28" t="n"/>
-      <c r="E36" s="28" t="n"/>
-      <c r="F36" s="29">
-        <f>IF(ABS(D22)&lt;=0.15,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="G36" s="14" t="n"/>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>Competitor avg ADR</t>
+        </is>
+      </c>
+      <c r="D31" s="27">
+        <f>AVERAGE(D26:D29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="19" customHeight="1">
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>Your planned ADR</t>
+        </is>
+      </c>
+      <c r="D32" s="27">
+        <f>'Assumptions'!D6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>Your ADR vs market</t>
+        </is>
+      </c>
+      <c r="D33" s="28">
+        <f>IFERROR('Assumptions'!D6/AVERAGE(D26:D29)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35" ht="24" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>LOCATION SCORING (WEIGHTED)</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="5" t="n"/>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Score /10</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Weighted</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr"/>
     </row>
     <row r="37" ht="19" customHeight="1">
       <c r="B37" s="7" t="inlineStr">
         <is>
+          <t>Footfall / visibility</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D37" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="E37" s="29">
+        <f>C37*D37</f>
+        <v/>
+      </c>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="n"/>
+    </row>
+    <row r="38" ht="19" customHeight="1">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Transport access</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D38" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E38" s="29">
+        <f>C38*D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="14" t="n"/>
+      <c r="G38" s="14" t="n"/>
+    </row>
+    <row r="39" ht="19" customHeight="1">
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Nearby demand drivers</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D39" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="E39" s="29">
+        <f>C39*D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="8" t="n"/>
+    </row>
+    <row r="40" ht="19" customHeight="1">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Competition density</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D40" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E40" s="29">
+        <f>C40*D40</f>
+        <v/>
+      </c>
+      <c r="F40" s="14" t="n"/>
+      <c r="G40" s="14" t="n"/>
+    </row>
+    <row r="41" ht="19" customHeight="1">
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Lease cost vs ADR</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D41" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E41" s="29">
+        <f>C41*D41</f>
+        <v/>
+      </c>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
+    </row>
+    <row r="42" ht="19" customHeight="1">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Planning / fit-out ease</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D42" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="E42" s="29">
+        <f>C42*D42</f>
+        <v/>
+      </c>
+      <c r="F42" s="14" t="n"/>
+      <c r="G42" s="14" t="n"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="30" t="inlineStr">
+        <is>
+          <t>Location score / 10</t>
+        </is>
+      </c>
+      <c r="E43" s="31">
+        <f>SUM(E37:E42)</f>
+        <v/>
+      </c>
+      <c r="F43" s="32">
+        <f>IF(E43="","",IF(E43&gt;=7,"🟢 On target",IF(E43&gt;=5,"🟡 Watch","🔴 Action")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45" ht="24" customHeight="1">
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>PHASE 0 GO / NO-GO GATE</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="5" t="n"/>
+    </row>
+    <row r="46" ht="19" customHeight="1">
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>SOM room-nights within capacity</t>
+        </is>
+      </c>
+      <c r="C46" s="20" t="n"/>
+      <c r="D46" s="20" t="n"/>
+      <c r="E46" s="20" t="n"/>
+      <c r="F46" s="33">
+        <f>IF(F8&lt;= ('Assumptions'!D5*365),"PASS","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="G46" s="8" t="n"/>
+    </row>
+    <row r="47" ht="19" customHeight="1">
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>ADR competitive (within ±15% of market)</t>
+        </is>
+      </c>
+      <c r="C47" s="20" t="n"/>
+      <c r="D47" s="20" t="n"/>
+      <c r="E47" s="20" t="n"/>
+      <c r="F47" s="33">
+        <f>IF(ABS(D33)&lt;=0.15,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="G47" s="14" t="n"/>
+    </row>
+    <row r="48" ht="19" customHeight="1">
+      <c r="B48" s="7" t="inlineStr">
+        <is>
           <t>Location score ≥ 7/10</t>
         </is>
       </c>
-      <c r="C37" s="28" t="n"/>
-      <c r="D37" s="28" t="n"/>
-      <c r="E37" s="28" t="n"/>
-      <c r="F37" s="29">
-        <f>IF(E32&gt;=7,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="G37" s="8" t="n"/>
-    </row>
-    <row r="38"/>
-    <row r="39" ht="22" customHeight="1">
-      <c r="B39" s="30" t="inlineStr">
+      <c r="C48" s="20" t="n"/>
+      <c r="D48" s="20" t="n"/>
+      <c r="E48" s="20" t="n"/>
+      <c r="F48" s="33">
+        <f>IF(E43&gt;=7,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="G48" s="8" t="n"/>
+    </row>
+    <row r="49"/>
+    <row r="50" ht="22" customHeight="1">
+      <c r="B50" s="34" t="inlineStr">
         <is>
           <t>ASSET-FORGE · LEANTA Turnkey Pack · Boutique Hotel · v1.0 · 04/06/2026 · Phase 0 of 6</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="23">
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="B50:K50"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="F17:G17"/>
     <mergeCell ref="B24:G24"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="B34:G34"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B2:K2"/>
     <mergeCell ref="B1:K1"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B39:K39"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B22:G22"/>
     <mergeCell ref="B11:G11"/>
-    <mergeCell ref="D21:E21"/>
   </mergeCells>
-  <conditionalFormatting sqref="F32">
+  <conditionalFormatting sqref="F43">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>ISNUMBER(SEARCH("On target",F32))</formula>
+      <formula>ISNUMBER(SEARCH("On target",F43))</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>ISNUMBER(SEARCH("Watch",F32))</formula>
+      <formula>ISNUMBER(SEARCH("Watch",F43))</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>ISNUMBER(SEARCH("Action",F32))</formula>
+      <formula>ISNUMBER(SEARCH("Action",F43))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F35">
+  <conditionalFormatting sqref="F46">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -1297,7 +1526,7 @@
       <formula>"REVIEW"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F36">
+  <conditionalFormatting sqref="F47">
     <cfRule type="cellIs" priority="6" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -1305,7 +1534,7 @@
       <formula>"REVIEW"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F37">
+  <conditionalFormatting sqref="F48">
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -1373,84 +1602,84 @@
       <c r="F4" s="5" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="B5" s="31" t="inlineStr">
+      <c r="B5" s="35" t="inlineStr">
         <is>
           <t>Rooms available</t>
         </is>
       </c>
-      <c r="D5" s="32" t="n">
+      <c r="D5" s="36" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="31" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>ADR — average daily rate</t>
         </is>
       </c>
-      <c r="D6" s="33" t="n">
+      <c r="D6" s="37" t="n">
         <v>135</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
+      <c r="F6" s="38" t="inlineStr">
         <is>
           <t>4★ boutique IE €110–180</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="B7" s="31" t="inlineStr">
+      <c r="B7" s="35" t="inlineStr">
         <is>
           <t>Occupancy</t>
         </is>
       </c>
-      <c r="D7" s="35" t="n">
+      <c r="D7" s="39" t="n">
         <v>0.72</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
+      <c r="F7" s="38" t="inlineStr">
         <is>
           <t>annualised; 65–80% typical</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="B8" s="31" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>RevPAR (ADR × occupancy)</t>
         </is>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="27">
         <f>'Assumptions'!D6*'Assumptions'!D7</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="B9" s="31" t="inlineStr">
+      <c r="B9" s="35" t="inlineStr">
         <is>
           <t>F&amp;B + other revenue (% of rooms)</t>
         </is>
       </c>
-      <c r="D9" s="35" t="n">
+      <c r="D9" s="39" t="n">
         <v>0.28</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="B10" s="31" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>Rooms revenue / yr</t>
         </is>
       </c>
-      <c r="D10" s="36">
+      <c r="D10" s="40">
         <f>'Assumptions'!D5*365*'Assumptions'!D8</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="B11" s="31" t="inlineStr">
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>Total revenue / yr</t>
         </is>
       </c>
-      <c r="D11" s="36">
+      <c r="D11" s="40">
         <f>'Assumptions'!D10*(1+'Assumptions'!D9)</f>
         <v/>
       </c>
@@ -1468,72 +1697,72 @@
       <c r="F13" s="5" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="B14" s="31" t="inlineStr">
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>Payroll (% of total revenue)</t>
         </is>
       </c>
-      <c r="D14" s="35" t="n">
+      <c r="D14" s="39" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="B15" s="31" t="inlineStr">
+      <c r="B15" s="35" t="inlineStr">
         <is>
           <t>F&amp;B cost (% of F&amp;B revenue)</t>
         </is>
       </c>
-      <c r="D15" s="35" t="n">
+      <c r="D15" s="39" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="B16" s="31" t="inlineStr">
+      <c r="B16" s="35" t="inlineStr">
         <is>
           <t>Rooms cost (% of rooms revenue)</t>
         </is>
       </c>
-      <c r="D16" s="35" t="n">
+      <c r="D16" s="39" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="31" t="inlineStr">
+      <c r="B17" s="35" t="inlineStr">
         <is>
           <t>Utilities (% of total revenue)</t>
         </is>
       </c>
-      <c r="D17" s="35" t="n">
+      <c r="D17" s="39" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="B18" s="31" t="inlineStr">
+      <c r="B18" s="35" t="inlineStr">
         <is>
           <t>Sales &amp; marketing (% of revenue)</t>
         </is>
       </c>
-      <c r="D18" s="35" t="n">
+      <c r="D18" s="39" t="n">
         <v>0.06</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="B19" s="31" t="inlineStr">
+      <c r="B19" s="35" t="inlineStr">
         <is>
           <t>Admin &amp; general (% of revenue)</t>
         </is>
       </c>
-      <c r="D19" s="35" t="n">
+      <c r="D19" s="39" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="B20" s="31" t="inlineStr">
+      <c r="B20" s="35" t="inlineStr">
         <is>
           <t>Property: rent/rates/insurance (%)</t>
         </is>
       </c>
-      <c r="D20" s="35" t="n">
+      <c r="D20" s="39" t="n">
         <v>0.12</v>
       </c>
     </row>
@@ -1550,92 +1779,92 @@
       <c r="F22" s="5" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="31" t="inlineStr">
+      <c r="B23" s="35" t="inlineStr">
         <is>
           <t>Lease deposit &amp; legal</t>
         </is>
       </c>
-      <c r="D23" s="37" t="n">
+      <c r="D23" s="41" t="n">
         <v>45000</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="B24" s="31" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr">
         <is>
           <t>Building refurbishment &amp; fit-out</t>
         </is>
       </c>
-      <c r="D24" s="37" t="n">
+      <c r="D24" s="41" t="n">
         <v>240000</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="B25" s="31" t="inlineStr">
+      <c r="B25" s="35" t="inlineStr">
         <is>
           <t>FF&amp;E (rooms, beds, furniture)</t>
         </is>
       </c>
-      <c r="D25" s="37" t="n">
+      <c r="D25" s="41" t="n">
         <v>120000</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="B26" s="31" t="inlineStr">
+      <c r="B26" s="35" t="inlineStr">
         <is>
           <t>Kitchen &amp; F&amp;B equipment</t>
         </is>
       </c>
-      <c r="D26" s="37" t="n">
+      <c r="D26" s="41" t="n">
         <v>55000</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="B27" s="31" t="inlineStr">
+      <c r="B27" s="35" t="inlineStr">
         <is>
           <t>IT, PMS, POS &amp; networking</t>
         </is>
       </c>
-      <c r="D27" s="37" t="n">
+      <c r="D27" s="41" t="n">
         <v>30000</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="B28" s="31" t="inlineStr">
+      <c r="B28" s="35" t="inlineStr">
         <is>
           <t>Branding, signage &amp; website</t>
         </is>
       </c>
-      <c r="D28" s="37" t="n">
+      <c r="D28" s="41" t="n">
         <v>25000</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="B29" s="31" t="inlineStr">
+      <c r="B29" s="35" t="inlineStr">
         <is>
           <t>Pre-opening payroll &amp; training</t>
         </is>
       </c>
-      <c r="D29" s="37" t="n">
+      <c r="D29" s="41" t="n">
         <v>35000</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="B30" s="31" t="inlineStr">
+      <c r="B30" s="35" t="inlineStr">
         <is>
           <t>Working capital buffer</t>
         </is>
       </c>
-      <c r="D30" s="37" t="n">
+      <c r="D30" s="41" t="n">
         <v>50000</v>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="25" t="inlineStr">
+      <c r="B31" s="30" t="inlineStr">
         <is>
           <t>Total capex required</t>
         </is>
       </c>
-      <c r="D31" s="36">
+      <c r="D31" s="40">
         <f>SUM(D23:D30)</f>
         <v/>
       </c>
@@ -1653,68 +1882,68 @@
       <c r="F33" s="5" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="B34" s="31" t="inlineStr">
+      <c r="B34" s="35" t="inlineStr">
         <is>
           <t>Founder equity (incl. SURE refund)</t>
         </is>
       </c>
-      <c r="D34" s="37" t="n">
+      <c r="D34" s="41" t="n">
         <v>180000</v>
       </c>
-      <c r="F34" s="38">
+      <c r="F34" s="42">
         <f>IF($D$34="","",D34/SUM($D$34:$D$37))</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="B35" s="31" t="inlineStr">
+      <c r="B35" s="35" t="inlineStr">
         <is>
           <t>LEO Priming grant</t>
         </is>
       </c>
-      <c r="D35" s="37" t="n">
+      <c r="D35" s="41" t="n">
         <v>80000</v>
       </c>
-      <c r="F35" s="38">
+      <c r="F35" s="42">
         <f>IF($D$35="","",D35/SUM($D$34:$D$37))</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="B36" s="31" t="inlineStr">
+      <c r="B36" s="35" t="inlineStr">
         <is>
           <t>Bank / SBCI term loan</t>
         </is>
       </c>
-      <c r="D36" s="37" t="n">
+      <c r="D36" s="41" t="n">
         <v>300000</v>
       </c>
-      <c r="F36" s="38">
+      <c r="F36" s="42">
         <f>IF($D$36="","",D36/SUM($D$34:$D$37))</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="B37" s="31" t="inlineStr">
+      <c r="B37" s="35" t="inlineStr">
         <is>
           <t>Microfinance Ireland loan</t>
         </is>
       </c>
-      <c r="D37" s="37" t="n">
+      <c r="D37" s="41" t="n">
         <v>40000</v>
       </c>
-      <c r="F37" s="38">
+      <c r="F37" s="42">
         <f>IF($D$37="","",D37/SUM($D$34:$D$37))</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="25" t="inlineStr">
+      <c r="B38" s="30" t="inlineStr">
         <is>
           <t>Total funding raised</t>
         </is>
       </c>
-      <c r="D38" s="36">
+      <c r="D38" s="40">
         <f>SUM(D34:D37)</f>
         <v/>
       </c>
@@ -1725,7 +1954,7 @@
           <t>Funding vs capex (surplus/gap)</t>
         </is>
       </c>
-      <c r="D39" s="36">
+      <c r="D39" s="40">
         <f>'Assumptions'!D38-'Assumptions'!D31</f>
         <v/>
       </c>
@@ -1745,21 +1974,21 @@
     <row r="42" ht="30" customHeight="1">
       <c r="B42" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ADR/occupancy/RevPAR benchmarks: Fáilte Ireland &amp; STR Ireland hotel performance reports (4-star/boutique ranges).</t>
+          <t xml:space="preserve">  ADR/occupancy/RevPAR: Fáilte Ireland Hotel Survey 2024 — 4★ ADR €143.50–€144.49, occupancy 60.2% (Dec) → 74.1% (Nov), RevPAR €86.42–€107.07.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Grant/funding figures: Local Enterprise Office (localenterprise.ie), Microfinance Ireland, SBCI, Fáilte Ireland investment schemes.</t>
+          <t xml:space="preserve">  Cost ratios: hospitality labour 25–35% of revenue (US long-run 31.2%); USALI F&amp;B cost-of-sales; GOP margin ~36–38% (HotelData 2025). See `startup_benchmarks` table.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="B44" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cost ratios (payroll ~30%, F&amp;B cost ~30%): USALI hotel P&amp;L conventions.</t>
+          <t xml:space="preserve">  Grant/funding figures: Local Enterprise Office (localenterprise.ie), Microfinance Ireland, SBCI, Fáilte Ireland investment schemes.</t>
         </is>
       </c>
     </row>
@@ -1772,7 +2001,7 @@
     </row>
     <row r="46"/>
     <row r="47" ht="22" customHeight="1">
-      <c r="B47" s="30" t="inlineStr">
+      <c r="B47" s="34" t="inlineStr">
         <is>
           <t>ASSET-FORGE · LEANTA Turnkey Pack · Boutique Hotel · v1.0 · 04/06/2026</t>
         </is>

</xml_diff>